<commit_message>
refactor: unify EX-GAS attribute source
</commit_message>
<xml_diff>
--- a/EX_GAS_Config/ProjectConfigTable/exgas_config/Datas/#exgas.attribute.xlsx
+++ b/EX_GAS_Config/ProjectConfigTable/exgas_config/Datas/#exgas.attribute.xlsx
@@ -1,12 +1,12 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="162913" fullCalcOnLoad="1"/>
@@ -502,12 +502,12 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Hp</t>
+          <t>Health</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>血量</t>
+          <t>生命</t>
         </is>
       </c>
       <c r="E4" s="2" t="n"/>
@@ -521,12 +521,12 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Mp</t>
+          <t>Mana</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>蓝量</t>
+          <t>法力</t>
         </is>
       </c>
       <c r="E5" s="2" t="n"/>
@@ -537,12 +537,12 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Spd</t>
+          <t>Agility</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>速度</t>
+          <t>敏捷</t>
         </is>
       </c>
     </row>
@@ -552,12 +552,12 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Atk</t>
+          <t>PhysicalAttack</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>攻击力</t>
+          <t>物理攻击</t>
         </is>
       </c>
     </row>
@@ -567,12 +567,12 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Def</t>
+          <t>PhysicalDefense</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>防御力</t>
+          <t>物理防御</t>
         </is>
       </c>
     </row>
@@ -582,7 +582,7 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Sp</t>
+          <t>Stamina</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
@@ -597,12 +597,12 @@
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>HpMax</t>
+          <t>MaxHealth</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>血上限</t>
+          <t>生命上限</t>
         </is>
       </c>
     </row>
@@ -612,12 +612,12 @@
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>MpMax</t>
+          <t>MaxMana</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>魔力上限</t>
+          <t>法力上限</t>
         </is>
       </c>
     </row>
@@ -627,7 +627,7 @@
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>SpMax</t>
+          <t>MaxStamina</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
@@ -642,7 +642,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>AtkRate</t>
+          <t>AttackRate</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -652,24 +652,64 @@
       </c>
     </row>
     <row r="14">
-      <c r="B14" s="2" t="n"/>
-      <c r="C14" s="2" t="n"/>
-      <c r="D14" s="2" t="n"/>
+      <c r="B14" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>MagicalAttack</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>法术攻击</t>
+        </is>
+      </c>
     </row>
     <row r="15">
-      <c r="B15" s="2" t="n"/>
-      <c r="C15" s="2" t="n"/>
-      <c r="D15" s="2" t="n"/>
+      <c r="B15" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>MagicalDefense</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>法术防御</t>
+        </is>
+      </c>
     </row>
     <row r="16">
-      <c r="B16" s="2" t="n"/>
-      <c r="C16" s="2" t="n"/>
-      <c r="D16" s="2" t="n"/>
+      <c r="B16" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>Luck</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>幸运</t>
+        </is>
+      </c>
     </row>
     <row r="17">
-      <c r="B17" s="2" t="n"/>
-      <c r="C17" s="2" t="n"/>
-      <c r="D17" s="2" t="n"/>
+      <c r="B17" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>AttackSpeed</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>攻击速度</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="B18" s="2" t="n"/>

</xml_diff>